<commit_message>
Handle uniform SKU batch pricing and keep browser open on errors
</commit_message>
<xml_diff>
--- a/examples/product-template/product-input-multisku.xlsx
+++ b/examples/product-template/product-input-multisku.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="147">
   <si>
     <t>ProductPilot 多SKU填写说明</t>
   </si>
@@ -1672,11 +1672,11 @@
       <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>19</v>
+      <c r="E2">
+        <v>146</v>
+      </c>
+      <c r="F2">
+        <v>188</v>
       </c>
       <c r="G2" t="s">
         <v>19</v>
@@ -1698,11 +1698,11 @@
       <c r="D3" t="s">
         <v>19</v>
       </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>19</v>
+      <c r="E3">
+        <v>146</v>
+      </c>
+      <c r="F3">
+        <v>188</v>
       </c>
       <c r="G3" t="s">
         <v>19</v>
@@ -1724,11 +1724,11 @@
       <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
+      <c r="E4">
+        <v>146</v>
+      </c>
+      <c r="F4">
+        <v>188</v>
       </c>
       <c r="G4" t="s">
         <v>19</v>
@@ -1750,11 +1750,11 @@
       <c r="D5" t="s">
         <v>19</v>
       </c>
-      <c r="E5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s">
-        <v>19</v>
+      <c r="E5">
+        <v>146</v>
+      </c>
+      <c r="F5">
+        <v>188</v>
       </c>
       <c r="G5" t="s">
         <v>19</v>
@@ -1776,11 +1776,11 @@
       <c r="D6" t="s">
         <v>19</v>
       </c>
-      <c r="E6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" t="s">
-        <v>19</v>
+      <c r="E6">
+        <v>146</v>
+      </c>
+      <c r="F6">
+        <v>188</v>
       </c>
       <c r="G6" t="s">
         <v>19</v>
@@ -1802,11 +1802,11 @@
       <c r="D7" t="s">
         <v>19</v>
       </c>
-      <c r="E7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" t="s">
-        <v>19</v>
+      <c r="E7">
+        <v>146</v>
+      </c>
+      <c r="F7">
+        <v>188</v>
       </c>
       <c r="G7" t="s">
         <v>19</v>
@@ -1828,11 +1828,11 @@
       <c r="D8" t="s">
         <v>19</v>
       </c>
-      <c r="E8" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" t="s">
-        <v>19</v>
+      <c r="E8">
+        <v>146</v>
+      </c>
+      <c r="F8">
+        <v>188</v>
       </c>
       <c r="G8" t="s">
         <v>19</v>
@@ -1854,11 +1854,11 @@
       <c r="D9" t="s">
         <v>19</v>
       </c>
-      <c r="E9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" t="s">
-        <v>19</v>
+      <c r="E9">
+        <v>146</v>
+      </c>
+      <c r="F9">
+        <v>188</v>
       </c>
       <c r="G9" t="s">
         <v>19</v>
@@ -1880,11 +1880,11 @@
       <c r="D10" t="s">
         <v>19</v>
       </c>
-      <c r="E10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" t="s">
-        <v>19</v>
+      <c r="E10">
+        <v>146</v>
+      </c>
+      <c r="F10">
+        <v>188</v>
       </c>
       <c r="G10" t="s">
         <v>19</v>
@@ -1906,11 +1906,11 @@
       <c r="D11" t="s">
         <v>19</v>
       </c>
-      <c r="E11" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" t="s">
-        <v>19</v>
+      <c r="E11">
+        <v>146</v>
+      </c>
+      <c r="F11">
+        <v>188</v>
       </c>
       <c r="G11" t="s">
         <v>19</v>
@@ -1932,11 +1932,11 @@
       <c r="D12" t="s">
         <v>19</v>
       </c>
-      <c r="E12" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" t="s">
-        <v>19</v>
+      <c r="E12">
+        <v>146</v>
+      </c>
+      <c r="F12">
+        <v>188</v>
       </c>
       <c r="G12" t="s">
         <v>19</v>
@@ -1958,11 +1958,11 @@
       <c r="D13" t="s">
         <v>19</v>
       </c>
-      <c r="E13" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" t="s">
-        <v>19</v>
+      <c r="E13">
+        <v>146</v>
+      </c>
+      <c r="F13">
+        <v>188</v>
       </c>
       <c r="G13" t="s">
         <v>19</v>
@@ -1984,11 +1984,11 @@
       <c r="D14" t="s">
         <v>19</v>
       </c>
-      <c r="E14" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" t="s">
-        <v>19</v>
+      <c r="E14">
+        <v>146</v>
+      </c>
+      <c r="F14">
+        <v>188</v>
       </c>
       <c r="G14" t="s">
         <v>19</v>
@@ -2010,11 +2010,11 @@
       <c r="D15" t="s">
         <v>19</v>
       </c>
-      <c r="E15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F15" t="s">
-        <v>19</v>
+      <c r="E15">
+        <v>146</v>
+      </c>
+      <c r="F15">
+        <v>188</v>
       </c>
       <c r="G15" t="s">
         <v>19</v>
@@ -2036,11 +2036,11 @@
       <c r="D16" t="s">
         <v>19</v>
       </c>
-      <c r="E16" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" t="s">
-        <v>19</v>
+      <c r="E16">
+        <v>146</v>
+      </c>
+      <c r="F16">
+        <v>188</v>
       </c>
       <c r="G16" t="s">
         <v>19</v>
@@ -2062,11 +2062,11 @@
       <c r="D17" t="s">
         <v>19</v>
       </c>
-      <c r="E17" t="s">
-        <v>19</v>
-      </c>
-      <c r="F17" t="s">
-        <v>19</v>
+      <c r="E17">
+        <v>146</v>
+      </c>
+      <c r="F17">
+        <v>188</v>
       </c>
       <c r="G17" t="s">
         <v>19</v>
@@ -2088,11 +2088,11 @@
       <c r="D18" t="s">
         <v>19</v>
       </c>
-      <c r="E18" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" t="s">
-        <v>19</v>
+      <c r="E18">
+        <v>146</v>
+      </c>
+      <c r="F18">
+        <v>188</v>
       </c>
       <c r="G18" t="s">
         <v>19</v>
@@ -2114,11 +2114,11 @@
       <c r="D19" t="s">
         <v>19</v>
       </c>
-      <c r="E19" t="s">
-        <v>19</v>
-      </c>
-      <c r="F19" t="s">
-        <v>19</v>
+      <c r="E19">
+        <v>146</v>
+      </c>
+      <c r="F19">
+        <v>188</v>
       </c>
       <c r="G19" t="s">
         <v>19</v>
@@ -2140,11 +2140,11 @@
       <c r="D20" t="s">
         <v>19</v>
       </c>
-      <c r="E20" t="s">
-        <v>19</v>
-      </c>
-      <c r="F20" t="s">
-        <v>19</v>
+      <c r="E20">
+        <v>146</v>
+      </c>
+      <c r="F20">
+        <v>188</v>
       </c>
       <c r="G20" t="s">
         <v>19</v>
@@ -2166,11 +2166,11 @@
       <c r="D21" t="s">
         <v>19</v>
       </c>
-      <c r="E21" t="s">
-        <v>19</v>
-      </c>
-      <c r="F21" t="s">
-        <v>19</v>
+      <c r="E21">
+        <v>146</v>
+      </c>
+      <c r="F21">
+        <v>188</v>
       </c>
       <c r="G21" t="s">
         <v>19</v>
@@ -2192,11 +2192,11 @@
       <c r="D22" t="s">
         <v>19</v>
       </c>
-      <c r="E22" t="s">
-        <v>19</v>
-      </c>
-      <c r="F22" t="s">
-        <v>19</v>
+      <c r="E22">
+        <v>146</v>
+      </c>
+      <c r="F22">
+        <v>188</v>
       </c>
       <c r="G22" t="s">
         <v>19</v>
@@ -2218,11 +2218,11 @@
       <c r="D23" t="s">
         <v>19</v>
       </c>
-      <c r="E23" t="s">
-        <v>19</v>
-      </c>
-      <c r="F23" t="s">
-        <v>19</v>
+      <c r="E23">
+        <v>146</v>
+      </c>
+      <c r="F23">
+        <v>188</v>
       </c>
       <c r="G23" t="s">
         <v>19</v>
@@ -2244,11 +2244,11 @@
       <c r="D24" t="s">
         <v>19</v>
       </c>
-      <c r="E24" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" t="s">
-        <v>19</v>
+      <c r="E24">
+        <v>146</v>
+      </c>
+      <c r="F24">
+        <v>188</v>
       </c>
       <c r="G24" t="s">
         <v>19</v>
@@ -2270,11 +2270,11 @@
       <c r="D25" t="s">
         <v>19</v>
       </c>
-      <c r="E25" t="s">
-        <v>19</v>
-      </c>
-      <c r="F25" t="s">
-        <v>19</v>
+      <c r="E25">
+        <v>146</v>
+      </c>
+      <c r="F25">
+        <v>188</v>
       </c>
       <c r="G25" t="s">
         <v>19</v>
@@ -2296,11 +2296,11 @@
       <c r="D26" t="s">
         <v>19</v>
       </c>
-      <c r="E26" t="s">
-        <v>19</v>
-      </c>
-      <c r="F26" t="s">
-        <v>19</v>
+      <c r="E26">
+        <v>146</v>
+      </c>
+      <c r="F26">
+        <v>188</v>
       </c>
       <c r="G26" t="s">
         <v>19</v>
@@ -2322,11 +2322,11 @@
       <c r="D27" t="s">
         <v>19</v>
       </c>
-      <c r="E27" t="s">
-        <v>19</v>
-      </c>
-      <c r="F27" t="s">
-        <v>19</v>
+      <c r="E27">
+        <v>146</v>
+      </c>
+      <c r="F27">
+        <v>188</v>
       </c>
       <c r="G27" t="s">
         <v>19</v>
@@ -2348,11 +2348,11 @@
       <c r="D28" t="s">
         <v>19</v>
       </c>
-      <c r="E28" t="s">
-        <v>19</v>
-      </c>
-      <c r="F28" t="s">
-        <v>19</v>
+      <c r="E28">
+        <v>146</v>
+      </c>
+      <c r="F28">
+        <v>188</v>
       </c>
       <c r="G28" t="s">
         <v>19</v>
@@ -2374,11 +2374,11 @@
       <c r="D29" t="s">
         <v>19</v>
       </c>
-      <c r="E29" t="s">
-        <v>19</v>
-      </c>
-      <c r="F29" t="s">
-        <v>19</v>
+      <c r="E29">
+        <v>146</v>
+      </c>
+      <c r="F29">
+        <v>188</v>
       </c>
       <c r="G29" t="s">
         <v>19</v>
@@ -2400,11 +2400,11 @@
       <c r="D30" t="s">
         <v>19</v>
       </c>
-      <c r="E30" t="s">
-        <v>19</v>
-      </c>
-      <c r="F30" t="s">
-        <v>19</v>
+      <c r="E30">
+        <v>146</v>
+      </c>
+      <c r="F30">
+        <v>188</v>
       </c>
       <c r="G30" t="s">
         <v>19</v>
@@ -2426,11 +2426,11 @@
       <c r="D31" t="s">
         <v>19</v>
       </c>
-      <c r="E31" t="s">
-        <v>19</v>
-      </c>
-      <c r="F31" t="s">
-        <v>19</v>
+      <c r="E31">
+        <v>146</v>
+      </c>
+      <c r="F31">
+        <v>188</v>
       </c>
       <c r="G31" t="s">
         <v>19</v>
@@ -2452,11 +2452,11 @@
       <c r="D32" t="s">
         <v>19</v>
       </c>
-      <c r="E32" t="s">
-        <v>19</v>
-      </c>
-      <c r="F32" t="s">
-        <v>19</v>
+      <c r="E32">
+        <v>146</v>
+      </c>
+      <c r="F32">
+        <v>188</v>
       </c>
       <c r="G32" t="s">
         <v>19</v>
@@ -2478,11 +2478,11 @@
       <c r="D33" t="s">
         <v>19</v>
       </c>
-      <c r="E33" t="s">
-        <v>19</v>
-      </c>
-      <c r="F33" t="s">
-        <v>19</v>
+      <c r="E33">
+        <v>146</v>
+      </c>
+      <c r="F33">
+        <v>188</v>
       </c>
       <c r="G33" t="s">
         <v>19</v>
@@ -2504,11 +2504,11 @@
       <c r="D34" t="s">
         <v>19</v>
       </c>
-      <c r="E34" t="s">
-        <v>19</v>
-      </c>
-      <c r="F34" t="s">
-        <v>19</v>
+      <c r="E34">
+        <v>146</v>
+      </c>
+      <c r="F34">
+        <v>188</v>
       </c>
       <c r="G34" t="s">
         <v>19</v>
@@ -2530,11 +2530,11 @@
       <c r="D35" t="s">
         <v>19</v>
       </c>
-      <c r="E35" t="s">
-        <v>19</v>
-      </c>
-      <c r="F35" t="s">
-        <v>19</v>
+      <c r="E35">
+        <v>146</v>
+      </c>
+      <c r="F35">
+        <v>188</v>
       </c>
       <c r="G35" t="s">
         <v>19</v>
@@ -2556,11 +2556,11 @@
       <c r="D36" t="s">
         <v>19</v>
       </c>
-      <c r="E36" t="s">
-        <v>19</v>
-      </c>
-      <c r="F36" t="s">
-        <v>19</v>
+      <c r="E36">
+        <v>146</v>
+      </c>
+      <c r="F36">
+        <v>188</v>
       </c>
       <c r="G36" t="s">
         <v>19</v>
@@ -2582,11 +2582,11 @@
       <c r="D37" t="s">
         <v>19</v>
       </c>
-      <c r="E37" t="s">
-        <v>19</v>
-      </c>
-      <c r="F37" t="s">
-        <v>19</v>
+      <c r="E37">
+        <v>146</v>
+      </c>
+      <c r="F37">
+        <v>188</v>
       </c>
       <c r="G37" t="s">
         <v>19</v>
@@ -2608,11 +2608,11 @@
       <c r="D38" t="s">
         <v>19</v>
       </c>
-      <c r="E38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F38" t="s">
-        <v>19</v>
+      <c r="E38">
+        <v>146</v>
+      </c>
+      <c r="F38">
+        <v>188</v>
       </c>
       <c r="G38" t="s">
         <v>19</v>
@@ -2634,11 +2634,11 @@
       <c r="D39" t="s">
         <v>19</v>
       </c>
-      <c r="E39" t="s">
-        <v>19</v>
-      </c>
-      <c r="F39" t="s">
-        <v>19</v>
+      <c r="E39">
+        <v>146</v>
+      </c>
+      <c r="F39">
+        <v>188</v>
       </c>
       <c r="G39" t="s">
         <v>19</v>
@@ -2660,11 +2660,11 @@
       <c r="D40" t="s">
         <v>19</v>
       </c>
-      <c r="E40" t="s">
-        <v>19</v>
-      </c>
-      <c r="F40" t="s">
-        <v>19</v>
+      <c r="E40">
+        <v>146</v>
+      </c>
+      <c r="F40">
+        <v>188</v>
       </c>
       <c r="G40" t="s">
         <v>19</v>
@@ -2686,11 +2686,11 @@
       <c r="D41" t="s">
         <v>19</v>
       </c>
-      <c r="E41" t="s">
-        <v>19</v>
-      </c>
-      <c r="F41" t="s">
-        <v>19</v>
+      <c r="E41">
+        <v>146</v>
+      </c>
+      <c r="F41">
+        <v>188</v>
       </c>
       <c r="G41" t="s">
         <v>19</v>
@@ -2712,11 +2712,11 @@
       <c r="D42" t="s">
         <v>19</v>
       </c>
-      <c r="E42" t="s">
-        <v>19</v>
-      </c>
-      <c r="F42" t="s">
-        <v>19</v>
+      <c r="E42">
+        <v>146</v>
+      </c>
+      <c r="F42">
+        <v>188</v>
       </c>
       <c r="G42" t="s">
         <v>19</v>
@@ -2738,11 +2738,11 @@
       <c r="D43" t="s">
         <v>19</v>
       </c>
-      <c r="E43" t="s">
-        <v>19</v>
-      </c>
-      <c r="F43" t="s">
-        <v>19</v>
+      <c r="E43">
+        <v>146</v>
+      </c>
+      <c r="F43">
+        <v>188</v>
       </c>
       <c r="G43" t="s">
         <v>19</v>
@@ -2764,11 +2764,11 @@
       <c r="D44" t="s">
         <v>19</v>
       </c>
-      <c r="E44" t="s">
-        <v>19</v>
-      </c>
-      <c r="F44" t="s">
-        <v>19</v>
+      <c r="E44">
+        <v>146</v>
+      </c>
+      <c r="F44">
+        <v>188</v>
       </c>
       <c r="G44" t="s">
         <v>19</v>
@@ -2790,11 +2790,11 @@
       <c r="D45" t="s">
         <v>19</v>
       </c>
-      <c r="E45" t="s">
-        <v>19</v>
-      </c>
-      <c r="F45" t="s">
-        <v>19</v>
+      <c r="E45">
+        <v>146</v>
+      </c>
+      <c r="F45">
+        <v>188</v>
       </c>
       <c r="G45" t="s">
         <v>19</v>
@@ -2816,11 +2816,11 @@
       <c r="D46" t="s">
         <v>19</v>
       </c>
-      <c r="E46" t="s">
-        <v>19</v>
-      </c>
-      <c r="F46" t="s">
-        <v>19</v>
+      <c r="E46">
+        <v>146</v>
+      </c>
+      <c r="F46">
+        <v>188</v>
       </c>
       <c r="G46" t="s">
         <v>19</v>
@@ -2842,11 +2842,11 @@
       <c r="D47" t="s">
         <v>19</v>
       </c>
-      <c r="E47" t="s">
-        <v>19</v>
-      </c>
-      <c r="F47" t="s">
-        <v>19</v>
+      <c r="E47">
+        <v>146</v>
+      </c>
+      <c r="F47">
+        <v>188</v>
       </c>
       <c r="G47" t="s">
         <v>19</v>
@@ -2868,11 +2868,11 @@
       <c r="D48" t="s">
         <v>19</v>
       </c>
-      <c r="E48" t="s">
-        <v>19</v>
-      </c>
-      <c r="F48" t="s">
-        <v>19</v>
+      <c r="E48">
+        <v>146</v>
+      </c>
+      <c r="F48">
+        <v>188</v>
       </c>
       <c r="G48" t="s">
         <v>19</v>
@@ -2894,11 +2894,11 @@
       <c r="D49" t="s">
         <v>19</v>
       </c>
-      <c r="E49" t="s">
-        <v>19</v>
-      </c>
-      <c r="F49" t="s">
-        <v>19</v>
+      <c r="E49">
+        <v>146</v>
+      </c>
+      <c r="F49">
+        <v>188</v>
       </c>
       <c r="G49" t="s">
         <v>19</v>
@@ -2920,11 +2920,11 @@
       <c r="D50" t="s">
         <v>19</v>
       </c>
-      <c r="E50" t="s">
-        <v>19</v>
-      </c>
-      <c r="F50" t="s">
-        <v>19</v>
+      <c r="E50">
+        <v>146</v>
+      </c>
+      <c r="F50">
+        <v>188</v>
       </c>
       <c r="G50" t="s">
         <v>19</v>
@@ -2946,11 +2946,11 @@
       <c r="D51" t="s">
         <v>19</v>
       </c>
-      <c r="E51" t="s">
-        <v>19</v>
-      </c>
-      <c r="F51" t="s">
-        <v>19</v>
+      <c r="E51">
+        <v>146</v>
+      </c>
+      <c r="F51">
+        <v>188</v>
       </c>
       <c r="G51" t="s">
         <v>19</v>
@@ -2972,11 +2972,11 @@
       <c r="D52" t="s">
         <v>19</v>
       </c>
-      <c r="E52" t="s">
-        <v>19</v>
-      </c>
-      <c r="F52" t="s">
-        <v>19</v>
+      <c r="E52">
+        <v>146</v>
+      </c>
+      <c r="F52">
+        <v>188</v>
       </c>
       <c r="G52" t="s">
         <v>19</v>
@@ -2998,11 +2998,11 @@
       <c r="D53" t="s">
         <v>19</v>
       </c>
-      <c r="E53" t="s">
-        <v>19</v>
-      </c>
-      <c r="F53" t="s">
-        <v>19</v>
+      <c r="E53">
+        <v>146</v>
+      </c>
+      <c r="F53">
+        <v>188</v>
       </c>
       <c r="G53" t="s">
         <v>19</v>
@@ -3024,11 +3024,11 @@
       <c r="D54" t="s">
         <v>19</v>
       </c>
-      <c r="E54" t="s">
-        <v>19</v>
-      </c>
-      <c r="F54" t="s">
-        <v>19</v>
+      <c r="E54">
+        <v>146</v>
+      </c>
+      <c r="F54">
+        <v>188</v>
       </c>
       <c r="G54" t="s">
         <v>19</v>
@@ -3050,11 +3050,11 @@
       <c r="D55" t="s">
         <v>19</v>
       </c>
-      <c r="E55" t="s">
-        <v>19</v>
-      </c>
-      <c r="F55" t="s">
-        <v>19</v>
+      <c r="E55">
+        <v>146</v>
+      </c>
+      <c r="F55">
+        <v>188</v>
       </c>
       <c r="G55" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Add product code support to draft automation
</commit_message>
<xml_diff>
--- a/examples/product-template/product-input-multisku.xlsx
+++ b/examples/product-template/product-input-multisku.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25860" windowHeight="19460" activeTab="2"/>
+    <workbookView windowWidth="25860" windowHeight="19460" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="填写说明" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="149">
   <si>
     <t>ProductPilot 多SKU填写说明</t>
   </si>
@@ -76,6 +76,9 @@
     <t>默认库存</t>
   </si>
   <si>
+    <t>商品编码</t>
+  </si>
+  <si>
     <t>SKU06</t>
   </si>
   <si>
@@ -91,34 +94,37 @@
     <t>146.64</t>
   </si>
   <si>
+    <t>demo001</t>
+  </si>
+  <si>
+    <t>颜色分类</t>
+  </si>
+  <si>
+    <t>鞋码</t>
+  </si>
+  <si>
+    <t>SKU名称</t>
+  </si>
+  <si>
+    <t>拼单价</t>
+  </si>
+  <si>
+    <t>单买价</t>
+  </si>
+  <si>
+    <t>参考价</t>
+  </si>
+  <si>
+    <t>库存</t>
+  </si>
+  <si>
+    <t>黑色</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>颜色分类</t>
-  </si>
-  <si>
-    <t>鞋码</t>
-  </si>
-  <si>
-    <t>SKU名称</t>
-  </si>
-  <si>
-    <t>拼单价</t>
-  </si>
-  <si>
-    <t>单买价</t>
-  </si>
-  <si>
-    <t>参考价</t>
-  </si>
-  <si>
-    <t>库存</t>
-  </si>
-  <si>
-    <t>黑色</t>
-  </si>
-  <si>
-    <t>38</t>
   </si>
   <si>
     <t>39</t>
@@ -1563,13 +1569,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="1" outlineLevelCol="7"/>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="1"/>
   <cols>
+    <col min="2" max="2" width="31.2941176470588" customWidth="1"/>
     <col min="4" max="4" width="29.5294117647059" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -1594,31 +1601,37 @@
       <c r="H1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" t="s">
         <v>19</v>
       </c>
-      <c r="G2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" t="s">
-        <v>19</v>
+      <c r="F2">
+        <v>150</v>
+      </c>
+      <c r="G2">
+        <v>180</v>
+      </c>
+      <c r="H2">
+        <v>1000</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1638,1455 +1651,807 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2">
-        <v>146</v>
-      </c>
-      <c r="F2">
-        <v>188</v>
-      </c>
-      <c r="G2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3">
-        <v>146</v>
-      </c>
-      <c r="F3">
-        <v>188</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4">
-        <v>146</v>
-      </c>
-      <c r="F4">
-        <v>188</v>
-      </c>
-      <c r="G4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5">
-        <v>146</v>
-      </c>
-      <c r="F5">
-        <v>188</v>
-      </c>
-      <c r="G5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6">
-        <v>146</v>
-      </c>
-      <c r="F6">
-        <v>188</v>
-      </c>
-      <c r="G6" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7">
-        <v>146</v>
-      </c>
-      <c r="F7">
-        <v>188</v>
-      </c>
-      <c r="G7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H7">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8">
-        <v>146</v>
-      </c>
-      <c r="F8">
-        <v>188</v>
-      </c>
-      <c r="G8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9">
-        <v>146</v>
-      </c>
-      <c r="F9">
-        <v>188</v>
-      </c>
-      <c r="G9" t="s">
-        <v>19</v>
-      </c>
-      <c r="H9">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10">
-        <v>146</v>
-      </c>
-      <c r="F10">
-        <v>188</v>
-      </c>
-      <c r="G10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11">
-        <v>146</v>
-      </c>
-      <c r="F11">
-        <v>188</v>
-      </c>
-      <c r="G11" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
         <v>34</v>
       </c>
-      <c r="C12" t="s">
-        <v>32</v>
-      </c>
       <c r="D12" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12">
-        <v>146</v>
-      </c>
-      <c r="F12">
-        <v>188</v>
-      </c>
-      <c r="G12" t="s">
-        <v>19</v>
-      </c>
-      <c r="H12">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13">
-        <v>146</v>
-      </c>
-      <c r="F13">
-        <v>188</v>
-      </c>
-      <c r="G13" t="s">
-        <v>19</v>
-      </c>
-      <c r="H13">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14">
-        <v>146</v>
-      </c>
-      <c r="F14">
-        <v>188</v>
-      </c>
-      <c r="G14" t="s">
-        <v>19</v>
-      </c>
-      <c r="H14">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D15" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15">
-        <v>146</v>
-      </c>
-      <c r="F15">
-        <v>188</v>
-      </c>
-      <c r="G15" t="s">
-        <v>19</v>
-      </c>
-      <c r="H15">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" t="s">
         <v>35</v>
       </c>
-      <c r="C16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16">
-        <v>146</v>
-      </c>
-      <c r="F16">
-        <v>188</v>
-      </c>
-      <c r="G16" t="s">
-        <v>19</v>
-      </c>
-      <c r="H16">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="D19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" t="s">
+        <v>33</v>
+      </c>
+      <c r="D23" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" t="s">
         <v>35</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" t="s">
         <v>31</v>
       </c>
-      <c r="D17" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17">
-        <v>146</v>
-      </c>
-      <c r="F17">
-        <v>188</v>
-      </c>
-      <c r="G17" t="s">
-        <v>19</v>
-      </c>
-      <c r="H17">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="D27" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" t="s">
+        <v>33</v>
+      </c>
+      <c r="D29" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D30" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>39</v>
+      </c>
+      <c r="C31" t="s">
         <v>35</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D31" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" t="s">
+        <v>29</v>
+      </c>
+      <c r="D32" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" t="s">
         <v>32</v>
       </c>
-      <c r="D18" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18">
-        <v>146</v>
-      </c>
-      <c r="F18">
-        <v>188</v>
-      </c>
-      <c r="G18" t="s">
-        <v>19</v>
-      </c>
-      <c r="H18">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="D34" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" t="s">
+        <v>33</v>
+      </c>
+      <c r="D35" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" t="s">
+        <v>34</v>
+      </c>
+      <c r="D36" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>30</v>
+      </c>
+      <c r="B37" t="s">
+        <v>40</v>
+      </c>
+      <c r="C37" t="s">
         <v>35</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D37" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" t="s">
+        <v>30</v>
+      </c>
+      <c r="B38" t="s">
+        <v>41</v>
+      </c>
+      <c r="C38" t="s">
+        <v>29</v>
+      </c>
+      <c r="D38" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>30</v>
+      </c>
+      <c r="B39" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" t="s">
+        <v>31</v>
+      </c>
+      <c r="D39" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>30</v>
+      </c>
+      <c r="B40" t="s">
+        <v>41</v>
+      </c>
+      <c r="C40" t="s">
+        <v>32</v>
+      </c>
+      <c r="D40" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>30</v>
+      </c>
+      <c r="B41" t="s">
+        <v>41</v>
+      </c>
+      <c r="C41" t="s">
         <v>33</v>
       </c>
-      <c r="D19" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19">
-        <v>146</v>
-      </c>
-      <c r="F19">
-        <v>188</v>
-      </c>
-      <c r="G19" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20">
-        <v>146</v>
-      </c>
-      <c r="F20">
-        <v>188</v>
-      </c>
-      <c r="G20" t="s">
-        <v>19</v>
-      </c>
-      <c r="H20">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D41" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>30</v>
+      </c>
+      <c r="B42" t="s">
+        <v>41</v>
+      </c>
+      <c r="C42" t="s">
+        <v>34</v>
+      </c>
+      <c r="D42" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>30</v>
+      </c>
+      <c r="B43" t="s">
+        <v>41</v>
+      </c>
+      <c r="C43" t="s">
+        <v>35</v>
+      </c>
+      <c r="D43" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" t="s">
+        <v>30</v>
+      </c>
+      <c r="B44" t="s">
+        <v>42</v>
+      </c>
+      <c r="C44" t="s">
         <v>29</v>
       </c>
-      <c r="D21" t="s">
-        <v>19</v>
-      </c>
-      <c r="E21">
-        <v>146</v>
-      </c>
-      <c r="F21">
-        <v>188</v>
-      </c>
-      <c r="G21" t="s">
-        <v>19</v>
-      </c>
-      <c r="H21">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22">
-        <v>146</v>
-      </c>
-      <c r="F22">
-        <v>188</v>
-      </c>
-      <c r="G22" t="s">
-        <v>19</v>
-      </c>
-      <c r="H22">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" t="s">
-        <v>36</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D44" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" t="s">
+        <v>30</v>
+      </c>
+      <c r="B45" t="s">
+        <v>42</v>
+      </c>
+      <c r="C45" t="s">
         <v>31</v>
       </c>
-      <c r="D23" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23">
-        <v>146</v>
-      </c>
-      <c r="F23">
-        <v>188</v>
-      </c>
-      <c r="G23" t="s">
-        <v>19</v>
-      </c>
-      <c r="H23">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24" t="s">
-        <v>36</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="D45" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" t="s">
+        <v>30</v>
+      </c>
+      <c r="B46" t="s">
+        <v>42</v>
+      </c>
+      <c r="C46" t="s">
         <v>32</v>
       </c>
-      <c r="D24" t="s">
-        <v>19</v>
-      </c>
-      <c r="E24">
-        <v>146</v>
-      </c>
-      <c r="F24">
-        <v>188</v>
-      </c>
-      <c r="G24" t="s">
-        <v>19</v>
-      </c>
-      <c r="H24">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" t="s">
-        <v>19</v>
-      </c>
-      <c r="B25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="D46" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B47" t="s">
+        <v>42</v>
+      </c>
+      <c r="C47" t="s">
         <v>33</v>
       </c>
-      <c r="D25" t="s">
-        <v>19</v>
-      </c>
-      <c r="E25">
-        <v>146</v>
-      </c>
-      <c r="F25">
-        <v>188</v>
-      </c>
-      <c r="G25" t="s">
-        <v>19</v>
-      </c>
-      <c r="H25">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B26" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" t="s">
-        <v>19</v>
-      </c>
-      <c r="E26">
-        <v>146</v>
-      </c>
-      <c r="F26">
-        <v>188</v>
-      </c>
-      <c r="G26" t="s">
-        <v>19</v>
-      </c>
-      <c r="H26">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" t="s">
-        <v>19</v>
-      </c>
-      <c r="B27" t="s">
-        <v>37</v>
-      </c>
-      <c r="C27" t="s">
-        <v>29</v>
-      </c>
-      <c r="D27" t="s">
-        <v>19</v>
-      </c>
-      <c r="E27">
-        <v>146</v>
-      </c>
-      <c r="F27">
-        <v>188</v>
-      </c>
-      <c r="G27" t="s">
-        <v>19</v>
-      </c>
-      <c r="H27">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
-      <c r="A28" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" t="s">
-        <v>37</v>
-      </c>
-      <c r="C28" t="s">
-        <v>30</v>
-      </c>
-      <c r="D28" t="s">
-        <v>19</v>
-      </c>
-      <c r="E28">
-        <v>146</v>
-      </c>
-      <c r="F28">
-        <v>188</v>
-      </c>
-      <c r="G28" t="s">
-        <v>19</v>
-      </c>
-      <c r="H28">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
-      <c r="A29" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" t="s">
-        <v>37</v>
-      </c>
-      <c r="C29" t="s">
-        <v>31</v>
-      </c>
-      <c r="D29" t="s">
-        <v>19</v>
-      </c>
-      <c r="E29">
-        <v>146</v>
-      </c>
-      <c r="F29">
-        <v>188</v>
-      </c>
-      <c r="G29" t="s">
-        <v>19</v>
-      </c>
-      <c r="H29">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" t="s">
-        <v>19</v>
-      </c>
-      <c r="B30" t="s">
-        <v>37</v>
-      </c>
-      <c r="C30" t="s">
-        <v>32</v>
-      </c>
-      <c r="D30" t="s">
-        <v>19</v>
-      </c>
-      <c r="E30">
-        <v>146</v>
-      </c>
-      <c r="F30">
-        <v>188</v>
-      </c>
-      <c r="G30" t="s">
-        <v>19</v>
-      </c>
-      <c r="H30">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
-      <c r="A31" t="s">
-        <v>19</v>
-      </c>
-      <c r="B31" t="s">
-        <v>37</v>
-      </c>
-      <c r="C31" t="s">
-        <v>33</v>
-      </c>
-      <c r="D31" t="s">
-        <v>19</v>
-      </c>
-      <c r="E31">
-        <v>146</v>
-      </c>
-      <c r="F31">
-        <v>188</v>
-      </c>
-      <c r="G31" t="s">
-        <v>19</v>
-      </c>
-      <c r="H31">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
-      <c r="A32" t="s">
-        <v>19</v>
-      </c>
-      <c r="B32" t="s">
-        <v>38</v>
-      </c>
-      <c r="C32" t="s">
-        <v>28</v>
-      </c>
-      <c r="D32" t="s">
-        <v>19</v>
-      </c>
-      <c r="E32">
-        <v>146</v>
-      </c>
-      <c r="F32">
-        <v>188</v>
-      </c>
-      <c r="G32" t="s">
-        <v>19</v>
-      </c>
-      <c r="H32">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
-      <c r="A33" t="s">
-        <v>19</v>
-      </c>
-      <c r="B33" t="s">
-        <v>38</v>
-      </c>
-      <c r="C33" t="s">
-        <v>29</v>
-      </c>
-      <c r="D33" t="s">
-        <v>19</v>
-      </c>
-      <c r="E33">
-        <v>146</v>
-      </c>
-      <c r="F33">
-        <v>188</v>
-      </c>
-      <c r="G33" t="s">
-        <v>19</v>
-      </c>
-      <c r="H33">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" t="s">
-        <v>19</v>
-      </c>
-      <c r="B34" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" t="s">
-        <v>30</v>
-      </c>
-      <c r="D34" t="s">
-        <v>19</v>
-      </c>
-      <c r="E34">
-        <v>146</v>
-      </c>
-      <c r="F34">
-        <v>188</v>
-      </c>
-      <c r="G34" t="s">
-        <v>19</v>
-      </c>
-      <c r="H34">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="A35" t="s">
-        <v>19</v>
-      </c>
-      <c r="B35" t="s">
-        <v>38</v>
-      </c>
-      <c r="C35" t="s">
-        <v>31</v>
-      </c>
-      <c r="D35" t="s">
-        <v>19</v>
-      </c>
-      <c r="E35">
-        <v>146</v>
-      </c>
-      <c r="F35">
-        <v>188</v>
-      </c>
-      <c r="G35" t="s">
-        <v>19</v>
-      </c>
-      <c r="H35">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
-      <c r="A36" t="s">
-        <v>19</v>
-      </c>
-      <c r="B36" t="s">
-        <v>38</v>
-      </c>
-      <c r="C36" t="s">
-        <v>32</v>
-      </c>
-      <c r="D36" t="s">
-        <v>19</v>
-      </c>
-      <c r="E36">
-        <v>146</v>
-      </c>
-      <c r="F36">
-        <v>188</v>
-      </c>
-      <c r="G36" t="s">
-        <v>19</v>
-      </c>
-      <c r="H36">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
-      <c r="A37" t="s">
-        <v>19</v>
-      </c>
-      <c r="B37" t="s">
-        <v>38</v>
-      </c>
-      <c r="C37" t="s">
-        <v>33</v>
-      </c>
-      <c r="D37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37">
-        <v>146</v>
-      </c>
-      <c r="F37">
-        <v>188</v>
-      </c>
-      <c r="G37" t="s">
-        <v>19</v>
-      </c>
-      <c r="H37">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
-      <c r="A38" t="s">
-        <v>19</v>
-      </c>
-      <c r="B38" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" t="s">
-        <v>28</v>
-      </c>
-      <c r="D38" t="s">
-        <v>19</v>
-      </c>
-      <c r="E38">
-        <v>146</v>
-      </c>
-      <c r="F38">
-        <v>188</v>
-      </c>
-      <c r="G38" t="s">
-        <v>19</v>
-      </c>
-      <c r="H38">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" t="s">
-        <v>19</v>
-      </c>
-      <c r="B39" t="s">
-        <v>39</v>
-      </c>
-      <c r="C39" t="s">
-        <v>29</v>
-      </c>
-      <c r="D39" t="s">
-        <v>19</v>
-      </c>
-      <c r="E39">
-        <v>146</v>
-      </c>
-      <c r="F39">
-        <v>188</v>
-      </c>
-      <c r="G39" t="s">
-        <v>19</v>
-      </c>
-      <c r="H39">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
-      <c r="A40" t="s">
-        <v>19</v>
-      </c>
-      <c r="B40" t="s">
-        <v>39</v>
-      </c>
-      <c r="C40" t="s">
-        <v>30</v>
-      </c>
-      <c r="D40" t="s">
-        <v>19</v>
-      </c>
-      <c r="E40">
-        <v>146</v>
-      </c>
-      <c r="F40">
-        <v>188</v>
-      </c>
-      <c r="G40" t="s">
-        <v>19</v>
-      </c>
-      <c r="H40">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
-      <c r="A41" t="s">
-        <v>19</v>
-      </c>
-      <c r="B41" t="s">
-        <v>39</v>
-      </c>
-      <c r="C41" t="s">
-        <v>31</v>
-      </c>
-      <c r="D41" t="s">
-        <v>19</v>
-      </c>
-      <c r="E41">
-        <v>146</v>
-      </c>
-      <c r="F41">
-        <v>188</v>
-      </c>
-      <c r="G41" t="s">
-        <v>19</v>
-      </c>
-      <c r="H41">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
-      <c r="A42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B42" t="s">
-        <v>39</v>
-      </c>
-      <c r="C42" t="s">
-        <v>32</v>
-      </c>
-      <c r="D42" t="s">
-        <v>19</v>
-      </c>
-      <c r="E42">
-        <v>146</v>
-      </c>
-      <c r="F42">
-        <v>188</v>
-      </c>
-      <c r="G42" t="s">
-        <v>19</v>
-      </c>
-      <c r="H42">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" t="s">
-        <v>19</v>
-      </c>
-      <c r="B43" t="s">
-        <v>39</v>
-      </c>
-      <c r="C43" t="s">
-        <v>33</v>
-      </c>
-      <c r="D43" t="s">
-        <v>19</v>
-      </c>
-      <c r="E43">
-        <v>146</v>
-      </c>
-      <c r="F43">
-        <v>188</v>
-      </c>
-      <c r="G43" t="s">
-        <v>19</v>
-      </c>
-      <c r="H43">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
-      <c r="A44" t="s">
-        <v>19</v>
-      </c>
-      <c r="B44" t="s">
-        <v>40</v>
-      </c>
-      <c r="C44" t="s">
-        <v>28</v>
-      </c>
-      <c r="D44" t="s">
-        <v>19</v>
-      </c>
-      <c r="E44">
-        <v>146</v>
-      </c>
-      <c r="F44">
-        <v>188</v>
-      </c>
-      <c r="G44" t="s">
-        <v>19</v>
-      </c>
-      <c r="H44">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
-      <c r="A45" t="s">
-        <v>19</v>
-      </c>
-      <c r="B45" t="s">
-        <v>40</v>
-      </c>
-      <c r="C45" t="s">
-        <v>29</v>
-      </c>
-      <c r="D45" t="s">
-        <v>19</v>
-      </c>
-      <c r="E45">
-        <v>146</v>
-      </c>
-      <c r="F45">
-        <v>188</v>
-      </c>
-      <c r="G45" t="s">
-        <v>19</v>
-      </c>
-      <c r="H45">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
-      <c r="A46" t="s">
-        <v>19</v>
-      </c>
-      <c r="B46" t="s">
-        <v>40</v>
-      </c>
-      <c r="C46" t="s">
-        <v>30</v>
-      </c>
-      <c r="D46" t="s">
-        <v>19</v>
-      </c>
-      <c r="E46">
-        <v>146</v>
-      </c>
-      <c r="F46">
-        <v>188</v>
-      </c>
-      <c r="G46" t="s">
-        <v>19</v>
-      </c>
-      <c r="H46">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
-      <c r="A47" t="s">
-        <v>19</v>
-      </c>
-      <c r="B47" t="s">
-        <v>40</v>
-      </c>
-      <c r="C47" t="s">
-        <v>31</v>
-      </c>
       <c r="D47" t="s">
-        <v>19</v>
-      </c>
-      <c r="E47">
-        <v>146</v>
-      </c>
-      <c r="F47">
-        <v>188</v>
-      </c>
-      <c r="G47" t="s">
-        <v>19</v>
-      </c>
-      <c r="H47">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B48" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C48" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D48" t="s">
-        <v>19</v>
-      </c>
-      <c r="E48">
-        <v>146</v>
-      </c>
-      <c r="F48">
-        <v>188</v>
-      </c>
-      <c r="G48" t="s">
-        <v>19</v>
-      </c>
-      <c r="H48">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B49" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C49" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D49" t="s">
-        <v>19</v>
-      </c>
-      <c r="E49">
-        <v>146</v>
-      </c>
-      <c r="F49">
-        <v>188</v>
-      </c>
-      <c r="G49" t="s">
-        <v>19</v>
-      </c>
-      <c r="H49">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B50" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C50" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E50">
-        <v>146</v>
-      </c>
-      <c r="F50">
-        <v>188</v>
-      </c>
-      <c r="G50" t="s">
-        <v>19</v>
-      </c>
-      <c r="H50">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B51" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C51" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D51" t="s">
-        <v>19</v>
-      </c>
-      <c r="E51">
-        <v>146</v>
-      </c>
-      <c r="F51">
-        <v>188</v>
-      </c>
-      <c r="G51" t="s">
-        <v>19</v>
-      </c>
-      <c r="H51">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B52" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C52" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D52" t="s">
-        <v>19</v>
-      </c>
-      <c r="E52">
-        <v>146</v>
-      </c>
-      <c r="F52">
-        <v>188</v>
-      </c>
-      <c r="G52" t="s">
-        <v>19</v>
-      </c>
-      <c r="H52">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B53" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C53" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D53" t="s">
-        <v>19</v>
-      </c>
-      <c r="E53">
-        <v>146</v>
-      </c>
-      <c r="F53">
-        <v>188</v>
-      </c>
-      <c r="G53" t="s">
-        <v>19</v>
-      </c>
-      <c r="H53">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B54" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C54" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D54" t="s">
-        <v>19</v>
-      </c>
-      <c r="E54">
-        <v>146</v>
-      </c>
-      <c r="F54">
-        <v>188</v>
-      </c>
-      <c r="G54" t="s">
-        <v>19</v>
-      </c>
-      <c r="H54">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B55" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C55" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D55" t="s">
-        <v>19</v>
-      </c>
-      <c r="E55">
-        <v>146</v>
-      </c>
-      <c r="F55">
-        <v>188</v>
-      </c>
-      <c r="G55" t="s">
-        <v>19</v>
-      </c>
-      <c r="H55">
-        <v>1000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B56" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C56" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D56" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E56" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F56" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="G56" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="H56" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -3109,302 +2474,302 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="B4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="B5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="B6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="B9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
         <v>52</v>
-      </c>
-      <c r="C10" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="B11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E18" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E19" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C21" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E21" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -3425,112 +2790,112 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -3547,322 +2912,322 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="50" spans="1:1">
       <c r="A50" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="51" spans="1:1">
       <c r="A51" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="52" spans="1:1">
       <c r="A52" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="58" spans="1:1">
       <c r="A58" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="59" spans="1:1">
       <c r="A59" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="60" spans="1:1">
       <c r="A60" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="61" spans="1:1">
       <c r="A61" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="62" spans="1:1">
       <c r="A62" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="63" spans="1:1">
       <c r="A63" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="64" spans="1:1">
       <c r="A64" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>